<commit_message>
feat(dga): close remaining Platforms Code gaps — icons, service page, date picker, accessibility page
- Unified SVG icon layer (dga-icons.js) replaces all Font Awesome icons
- Course page restructured to the DGA service-page template (details card,
  steps, requirements, required documents, service description)
- Platforms Code date picker (dga-datepicker.js) with Selected/Today/Prev-Next
- Built-in accessibility statement fallback; unknown page slugs now 404
- Single <main> landmark per page (nested mains in 20 views converted)
- Compliance form + evidence screenshots updated (161 full / 5 partial / 17 N/A)

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/dga/نموذج الالتزام - منصة الشهادات الاحترافية - جامعة شقراء.xlsx
+++ b/docs/dga/نموذج الالتزام - منصة الشهادات الاحترافية - جامعة شقراء.xlsx
@@ -1796,21 +1796,25 @@
       <c r="F20" s="149" t="n"/>
       <c r="G20" s="133" t="inlineStr">
         <is>
-          <t>تطبيق جزئي</t>
-        </is>
-      </c>
-      <c r="H20" s="45" t="n"/>
+          <t>تطبيق كلي</t>
+        </is>
+      </c>
+      <c r="H20" s="150" t="inlineStr">
+        <is>
+          <t>public/website/js/dga-icons.js</t>
+        </is>
+      </c>
       <c r="I20" s="152" t="inlineStr">
         <is>
-          <t>الأيقونات خطية (stroke) بأحجام 16/20/24px وبألوان محايدة، وألوان الحالات للتنبيهات فقط، والأيقونات الكبيرة بصيغة Featured icon (48px بخلفية خفيفة).</t>
-        </is>
-      </c>
-      <c r="J20" s="61" t="n"/>
-      <c r="K20" s="151" t="inlineStr">
-        <is>
-          <t>ما زالت بعض الصفحات الداخلية تستخدم خط الأيقونات القديم (Font Awesome)؛ استبدالها الكامل بمكتبة أيقونات كود المنصات مجدول في المرحلة التالية.</t>
-        </is>
-      </c>
+          <t>مكتبة أيقونات موحدة: جميع الأيقونات خطية SVG (stroke 2px) بأحجام 16/20/24px وبألوان محايدة، وألوان الحالات للتنبيهات فقط، والأيقونات الكبيرة بصيغة Featured icon (48px بخلفية خفيفة). طبقة dga-icons.js تستبدل أي أيقونة قديمة (Font Awesome) تلقائياً بأيقونة المكتبة الموحدة دون تغيير الحجم أو اللون.</t>
+        </is>
+      </c>
+      <c r="J20" s="156" t="inlineStr">
+        <is>
+          <t>docs/dga/screenshots/course-service-page.png</t>
+        </is>
+      </c>
+      <c r="K20" s="89" t="n"/>
     </row>
     <row r="21" ht="50.1" customHeight="1" s="95">
       <c r="C21" s="19" t="n"/>
@@ -1827,13 +1831,13 @@
       <c r="F21" s="131" t="n"/>
       <c r="G21" s="133" t="inlineStr">
         <is>
-          <t>تطبيق جزئي</t>
+          <t>تطبيق كلي</t>
         </is>
       </c>
       <c r="H21" s="131" t="n"/>
       <c r="I21" s="152" t="inlineStr">
         <is>
-          <t>الأيقونات الجديدة SVG خطية موحدة الحجم واللون؛ الصفحات القديمة ما زالت تستخدم Font Awesome.</t>
+          <t>مكتبة أيقونات واحدة (SVG خطية) في كل الصفحات؛ لم يتبقَّ أي استخدام لخط الأيقونات القديم في واجهات الزائر (تم التحقق آلياً: 0 عنصر Font Awesome بعد التحميل).</t>
         </is>
       </c>
       <c r="J21" s="94" t="n"/>
@@ -2118,21 +2122,25 @@
       <c r="F31" s="149" t="n"/>
       <c r="G31" s="133" t="inlineStr">
         <is>
-          <t>تطبيق جزئي</t>
-        </is>
-      </c>
-      <c r="H31" s="45" t="n"/>
+          <t>تطبيق كلي</t>
+        </is>
+      </c>
+      <c r="H31" s="150" t="inlineStr">
+        <is>
+          <t>app/Application/views/website/courses/page.blade.php</t>
+        </is>
+      </c>
       <c r="I31" s="152" t="inlineStr">
         <is>
-          <t>صفحة الدورة تحتوي على بطاقة تفاصيل الخدمة (السعر/المدة/المحاضرات) وزر إجرائي وتقييم وتغذية راجعة.</t>
-        </is>
-      </c>
-      <c r="J31" s="61" t="n"/>
-      <c r="K31" s="151" t="inlineStr">
-        <is>
-          <t>توحيد مسميات الأقسام (الخطوات، الشروط، المستندات المطلوبة، بطاقة تفاصيل الخدمة) في صفحة الدورة مجدول في المرحلة التالية.</t>
-        </is>
-      </c>
+          <t>صفحة الدورة (الخدمة) مبنية على قالب صفحة الخدمة: مسار تصفح، بطاقة تفاصيل الخدمة، وصف الخدمة، الخطوات، الشروط، المستندات المطلوبة، المحتوى، المدرب، التقييم والتغذية الراجعة، مع زر إجرائي ثابت.</t>
+        </is>
+      </c>
+      <c r="J31" s="156" t="inlineStr">
+        <is>
+          <t>docs/dga/screenshots/course-service-page.png</t>
+        </is>
+      </c>
+      <c r="K31" s="89" t="n"/>
     </row>
     <row r="32" ht="93" customHeight="1" s="95">
       <c r="C32" s="19" t="n"/>
@@ -2149,13 +2157,13 @@
       <c r="F32" s="131" t="n"/>
       <c r="G32" s="133" t="inlineStr">
         <is>
-          <t>تطبيق جزئي</t>
+          <t>تطبيق كلي</t>
         </is>
       </c>
       <c r="H32" s="131" t="n"/>
       <c r="I32" s="151" t="inlineStr">
         <is>
-          <t>المصطلحات الحالية: "محتوى الدورة"، "عن المدرب"، "التقييمات"؛ يجري توحيدها مع قالب صفحة الخدمة.</t>
+          <t>العناوين والمصطلحات مطابقة للقالب: "بطاقة تفاصيل الخدمة" (اسم الخدمة، التصنيف، المدة، عدد المحاضرات، اللغة، الرسوم، الشهادة، قناة التقديم، المستفيدون)، "وصف الخدمة"، "الخطوات" (4 خطوات بمكون Steps)، "الشروط"، "المستندات المطلوبة".</t>
         </is>
       </c>
       <c r="J32" s="94" t="n"/>
@@ -5359,23 +5367,22 @@
       </c>
       <c r="G146" s="133" t="inlineStr">
         <is>
-          <t>تطبيق جزئي</t>
+          <t>تطبيق كلي</t>
         </is>
       </c>
       <c r="H146" s="150" t="inlineStr">
         <is>
-          <t>public/website/css/front/dga-platforms-code.css §6</t>
+          <t>public/website/js/dga-datepicker.js + public/website/css/front/dga-platforms-code.css §27</t>
         </is>
       </c>
       <c r="I146" s="152" t="inlineStr">
         <is>
-          <t>حقول التاريخ بنمط حقل الإدخال وحالاته.</t>
-        </is>
-      </c>
-      <c r="J146" s="66" t="n"/>
-      <c r="K146" s="152" t="inlineStr">
-        <is>
-          <t>التقويم المنسدل يعتمد على المتصفح؛ مكون التقويم المعتمد (Selected/Today/Next-Prev) مجدول في المرحلة التالية.</t>
+          <t>مكون محدد التاريخ وفق كود المنصات: حقل إدخال بزر تقويم، ونافذة تقويم منبثقة بشبكة الأيام وأزرار الشهر السابق/التالي وأزرار اليوم/مسح، مع دعم لوحة المفاتيح وقارئ الشاشة.</t>
+        </is>
+      </c>
+      <c r="J146" s="163" t="inlineStr">
+        <is>
+          <t>docs/dga/screenshots/datepicker.png</t>
         </is>
       </c>
     </row>
@@ -5446,13 +5453,13 @@
       <c r="F149" s="131" t="n"/>
       <c r="G149" s="52" t="inlineStr">
         <is>
-          <t>تطبيق جزئي</t>
+          <t>تطبيق كلي</t>
         </is>
       </c>
       <c r="H149" s="56" t="n"/>
       <c r="I149" s="154" t="inlineStr">
         <is>
-          <t>حالات التقويم (Selected/Today/Next-Prev) بتصميم المتصفح الافتراضي حالياً.</t>
+          <t>Selected (خلفية أساسية ونص أبيض)، Today (إطار أساسي)، Next/Prev (أزرار 36px بحدود)، والأيام خارج النطاق Disabled.</t>
         </is>
       </c>
       <c r="J149" s="84" t="n"/>

</xml_diff>

<commit_message>
feat(dga): adopt the Platforms Code icon library (Hugeicons) on every page and component
- Hugeicons stroke-rounded (MIT, @hugeicons/core-free-icons) — the library used by
  the DGA Platforms Code and the approved su.edu.sa theme
- Server-side dgaIcon() helper + PHP map; JS map + dga-icons.js maps all legacy
  Font Awesome names and <i class="hgi hgi-*"> placeholders to the same library
- All hand-written inline SVGs in templates (stamp, header, footer, breadcrumbs,
  pagination, services, course service template, forms, filters, sitemap, errors …)
  replaced with library icons; course page PNG picture-icons and emoji replaced
- Date picker, select caret, external-link and search glyphs switched to the library
- Verified on 28 URLs: 0 Font Awesome, 0 custom SVGs, all icons square; asset v4.0

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/dga/نموذج الالتزام - منصة الشهادات الاحترافية - جامعة شقراء.xlsx
+++ b/docs/dga/نموذج الالتزام - منصة الشهادات الاحترافية - جامعة شقراء.xlsx
@@ -1805,12 +1805,12 @@
       </c>
       <c r="H20" s="150" t="inlineStr">
         <is>
-          <t>public/website/js/dga-icons.js</t>
+          <t>app/Application/Helpers/dga-icons-map.php + public/website/js/dga-hgi-map.js</t>
         </is>
       </c>
       <c r="I20" s="153" t="inlineStr">
         <is>
-          <t>مكتبة أيقونات موحدة: جميع الأيقونات خطية SVG (stroke 2px) بأحجام 16/20/24px وبألوان محايدة، وألوان الحالات للتنبيهات فقط، والأيقونات الكبيرة بصيغة Featured icon (48px بخلفية خفيفة). طبقة dga-icons.js تستبدل أي أيقونة قديمة (Font Awesome) تلقائياً بأيقونة المكتبة الموحدة دون تغيير الحجم أو اللون.</t>
+          <t>مكتبة الأيقونات المعتمدة في كود المنصات (Hugeicons – Stroke Rounded)، وهي نفس المكتبة المستخدمة في موقع جامعة شقراء المعتمد من الهيئة (su.edu.sa). جميع الأيقونات تُرسم من المكتبة عبر الدالة dgaIcon() في القوالب، وطبقة dga-icons.js تستبدل أي أيقونة قديمة (Font Awesome) تلقائياً بأيقونة المكتبة نفسها بالأحجام 16/20/24px وبألوان محايدة، وألوان الحالات للتنبيهات فقط.</t>
         </is>
       </c>
       <c r="J20" s="152" t="inlineStr">
@@ -1841,7 +1841,7 @@
       <c r="H21" s="131" t="n"/>
       <c r="I21" s="153" t="inlineStr">
         <is>
-          <t>مكتبة أيقونات واحدة (SVG خطية) في كل الصفحات؛ لم يتبقَّ أي استخدام لخط الأيقونات القديم في واجهات الزائر (تم التحقق آلياً: 0 عنصر Font Awesome بعد التحميل).</t>
+          <t>مكتبة واحدة (Hugeicons) في كل الصفحات دون تعديل في الشكل أو السماكة (1.5px) أو اللون؛ تم التحقق آلياً على 28 صفحة: 0 عنصر Font Awesome و0 أيقونات مخصصة بعد التحميل.</t>
         </is>
       </c>
       <c r="J21" s="94" t="n"/>

</xml_diff>